<commit_message>
Điền nội dung thật cho memo quyết định và dashboard v1/v2; bổ sung bảng thành viên
- memo/memo_quyet_dinh.md: từ khung trống sang bản đầy đủ 5 phần, khớp với README
- dashboard_hanh_dong_v2.xlsx: điền toàn bộ 9 sheet (phạm vi, chẩn đoán, nguyên nhân
  gốc, workflow AS-IS/TO-BE, lộ trình 30-60-90, chỉ số, quyết định, thay đổi v1->v2)
- dashboard_hanh_dong_v1.xlsx: điền bản nháp trước phản biện để có căn cứ đối chiếu
  ≥2 thay đổi thật giữa v1 và v2 (trước đây v1 và v2 gần như là cùng 1 template rỗng)
- README.md: thêm mục 0 (bảng thành viên, đang thiếu hoàn toàn) và sửa mục 7 để
  không còn nhắc tới "Option A/B/C" chưa từng được định nghĩa ở đâu trong bài
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -646,7 +646,11 @@
           <t>Sản phẩm AI (đúng 1)</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>VLearn — trợ lý hỗ trợ learner khi làm bài lab</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
@@ -655,7 +659,11 @@
           <t>Nhóm người dùng chính (đúng 1)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Learner đang học lab, đã từng bị kẹt và phải tự xoay xở trong 7 ngày gần đây</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
@@ -664,7 +672,11 @@
           <t>Quy trình trong phạm vi #1</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Gặp điểm kẹt (lỗi cài đặt môi trường ở bước 3 của bài lab)</t>
+        </is>
+      </c>
       <c r="C6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -673,7 +685,11 @@
           <t>Quy trình trong phạm vi #2</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Hỏi trợ lý AI tutor tích hợp</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -682,7 +698,11 @@
           <t>Quy trình trong phạm vi #3 (tuỳ chọn)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm chứng câu trả lời trước khi làm theo</t>
+        </is>
+      </c>
       <c r="C8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -691,7 +711,11 @@
           <t>Quy trình trong phạm vi #4 (tuỳ chọn)</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định đi tiếp hoặc chuyển sang hỏi lab coach</t>
+        </is>
+      </c>
       <c r="C9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
@@ -700,7 +724,11 @@
           <t>NGOÀI phạm vi (loại trừ rõ)</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Rollout toàn khoá học; để AI tự phán đoán đúng/sai thay learner; các điểm kẹt ngoài lỗi cài đặt môi trường ở bước 3</t>
+        </is>
+      </c>
       <c r="C10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
@@ -709,7 +737,11 @@
           <t>Triệu chứng quan sát được</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Learner rời nền tảng đi hỏi AI ngoài (Claude/ChatGPT) dù đã có AI tutor tích hợp; tự nói "buộc phải tin" vì không kiểm chứng được</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -718,7 +750,11 @@
           <t>Mức độ hiện tại (Usage / Pilot / Deployment / Adoption / Normalization)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Usage — đã dùng AI tutor tích hợp nhưng vẫn rời nền tảng để tự kiểm chứng; chưa vào Pilot có kiểm soát</t>
+        </is>
+      </c>
       <c r="C12" s="7" t="inlineStr"/>
     </row>
   </sheetData>
@@ -788,8 +824,16 @@
           <t>Workflow: AI nằm ở bước nào, đã đổi cách làm chưa?</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>AI tutor nằm ngoài luồng xử lý điểm kẹt chính thức; chưa có bước bàn giao khi AI không đủ căn cứ</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Learner rời nền tảng đi hỏi AI ngoài dù tutor tích hợp đã trả lời trước đó</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
@@ -801,8 +845,16 @@
           <t>Con người: ai dùng, ai né, vì sao?</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Learner vẫn dùng nhưng không tin kết quả; né bằng cách đi hỏi AI ngoài hoặc đồng đội</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Phỏng vấn: "Anh chụp slide lên... anh buộc phải tin thôi"</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -814,8 +866,16 @@
           <t>Mức sẵn sàng: dữ liệu / quyền / governance / kỹ năng / ngân sách?</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Tài liệu lab có nhưng không có người phụ trách cập nhật + lịch review</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Không tìm thấy owner tài liệu trong quy trình hiện tại</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -827,8 +887,16 @@
           <t>Độ tin cậy: câu trả lời có nguồn, ngày cập nhật, cách báo lỗi?</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Câu trả lời không tách được ý nào có nguồn trong tài liệu, ý nào AI tự suy luận</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Learner: "buộc phải tin thôi" — không có nguồn/ngày cập nhật đi kèm câu trả lời</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -840,8 +908,16 @@
           <t>Cách đo lường: đang đo gì, chỉ số có dẫn tới quyết định không?</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Đang đo lượt mở trợ giúp (activity); chưa đo tỷ lệ có nguồn, tỷ lệ làm lại hay kết quả hoàn thành bài lab</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard v1 chỉ có 2 chỉ số: lượt mở trợ giúp + thời gian tiết kiệm tự khai</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="inlineStr"/>
     </row>
     <row r="11">
@@ -880,9 +956,21 @@
           <t>Direction — hướng đi rõ chưa</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr"/>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Mục tiêu rõ: giảm thời gian bị kẹt, tăng tỷ lệ tự vượt qua bước 3 mà không bỏ lab</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Đủ điều kiện chạy pilot nhỏ</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -891,9 +979,21 @@
           <t>Readiness — dữ liệu, quyền, governance, kỹ năng, ngân sách</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>THIẾU</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Tài liệu lab thiếu owner + lịch cập nhật; chưa có nhãn phân biệt nguồn trong/ngoài tài liệu</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Pilot phải sửa readiness (gắn nguồn, chỉ định data owner) trước khi mở rộng</t>
+        </is>
+      </c>
       <c r="E14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -902,9 +1002,21 @@
           <t>Absorption — owner, hỗ trợ vận hành, cơ chế học từ lỗi</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr"/>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>THIẾU</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Chưa có owner vận hành chất lượng câu trả lời; chưa có kênh chuyển coach rõ ràng</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Cần lập QA owner + đường chuyển coach trong 30 ngày đầu trước khi tính mở rộng</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -939,8 +1051,16 @@
           <t>Người giữ quyền (phê duyệt cuối, ngoại lệ)</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr"/>
-      <c r="C19" s="7" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Phê duyệt learner có đủ điều kiện đi tiếp bài lab hay cần chuyển coach</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Lab coach</t>
+        </is>
+      </c>
       <c r="D19" s="7" t="inlineStr"/>
       <c r="E19" s="7" t="inlineStr"/>
     </row>
@@ -950,8 +1070,16 @@
           <t>AI hỗ trợ — người kiểm (tìm / tóm tắt / tạo nháp)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr"/>
-      <c r="C20" s="7" t="inlineStr"/>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Tìm đoạn tài liệu liên quan, tóm tắt hướng xử lý điểm kẹt, gắn nguồn + ngày cập nhật</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>AI tutor; learner tự kiểm chứng trước khi làm theo</t>
+        </is>
+      </c>
       <c r="D20" s="7" t="inlineStr"/>
       <c r="E20" s="7" t="inlineStr"/>
     </row>
@@ -961,8 +1089,16 @@
           <t>AI tự động (lặp lại, rủi ro thấp, có tiêu chí kiểm tra)</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr"/>
-      <c r="C21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Không áp dụng ở giai đoạn pilot — chưa đủ dữ liệu QA để tự động hoá</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Không có (giữ nguyên có người kiểm ở mọi bước cho tới khi QA đạt ngưỡng)</t>
+        </is>
+      </c>
       <c r="D21" s="7" t="inlineStr"/>
       <c r="E21" s="7" t="inlineStr"/>
     </row>
@@ -1006,10 +1142,26 @@
           <t>Awareness — biết có công cụ</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr"/>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
-      <c r="E25" s="7" t="inlineStr"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Learner không biết AI tutor có thể xử lý loại lỗi cài đặt này</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Learner đi hỏi AI ngoài trước khi thử tutor tích hợp trong 2/3 phiên quan sát</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Ghi rõ trong màn hình lỗi: "Hỏi AI tutor" là bước đầu tiên khi kẹt ở bước 3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -1017,10 +1169,26 @@
           <t>Desire — muốn dùng / tin tưởng</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr"/>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr"/>
-      <c r="E26" s="7" t="inlineStr"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Ngại tin câu trả lời vì không thấy nguồn, thấy ngày cập nhật</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>"Anh buộc phải tin thôi" — không kiểm chứng được nên không dám làm theo</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Thêm trích nguồn + ngày cập nhật vào mọi câu trả lời, không mở lớp đào tạo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -1028,10 +1196,26 @@
           <t>Knowledge — biết cách dùng</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr"/>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr"/>
-      <c r="E27" s="7" t="inlineStr"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Chưa biết cách đọc nguồn được trích và khi nào nên chuyển coach</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Learner không thử bước kiểm chứng, đi thẳng sang hỏi người/AI ngoài</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Thêm hướng dẫn ngắn ngay tại màn hình trả lời, không phải khoá học riêng</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1039,10 +1223,26 @@
           <t>Ability — làm được trong việc thật</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr"/>
-      <c r="C28" s="7" t="inlineStr"/>
-      <c r="D28" s="7" t="inlineStr"/>
-      <c r="E28" s="7" t="inlineStr"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Chưa từng thực hành luồng hỏi AI → xem nguồn → kiểm chứng → đi tiếp/chuyển coach trong bài lab thật</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Chưa có dữ liệu learner hoàn thành đủ luồng mới</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Đưa luồng mới vào đúng bước 3 của pilot, đo trong 0–30 ngày</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -1050,10 +1250,26 @@
           <t>Reinforcement — được củng cố, không quay lại cách cũ</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr"/>
-      <c r="C29" s="7" t="inlineStr"/>
-      <c r="D29" s="7" t="inlineStr"/>
-      <c r="E29" s="7" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Không có phản hồi lỗi hay theo dõi hành vi mới nên dễ quay lại cách cũ (hỏi người/AI ngoài)</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard v1 không đo hành vi làm lại hay tỷ lệ chuyển coach thành công</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung chỉ số hành vi + rủi ro/bàn giao vào dashboard v2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1066,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1138,11 +1354,54 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Độ tin cậy không được thiết kế trong lượt trả lời — learner không biết ý nào có nguồn, ý nào không</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>5 câu hỏi chẩn đoán (trục Tin cậy) + ADKAR (Desire)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Phỏng vấn learner: "Anh chụp slide lên... anh buộc phải tin thôi" — không kiểm chứng được nên buộc phải tin</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Learner dùng thử rồi quay lại hỏi người/AI ngoài</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Workflow không có đường bàn giao ít ma sát sang coach khi AI không đủ căn cứ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5 câu hỏi chẩn đoán (trục Workflow) + Mollick (bàn giao người–AI)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Quan sát: learner rời nền tảng đi hỏi AI ngoài (Claude/ChatGPT) dù đã thử AI tutor tích hợp trước</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dashboard chỉ thấy "lượt dùng thấp", không thấy vì sao</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1238,12 +1497,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Gặp điểm kẹt ở bước 3 (cài đặt môi trường)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Learner tự tìm, hỏi AI ngoài hoặc đồng đội — không rõ ai chịu trách nhiệm câu trả lời</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Hỏi AI tutor tích hợp → xem nguồn tài liệu + ngày cập nhật → kiểm chứng → đi tiếp hoặc chuyển coach</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Tài liệu bài lab bước 3 (có owner + lịch cập nhật)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Lab coach trực pilot</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>AI trả lời không tìm thấy nguồn trong tài liệu → tự gắn nhãn "không đủ căn cứ" → chuyển coach trong ca trực</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr"/>
@@ -1382,7 +1665,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>&lt;tên&gt;</t>
+          <t>Product owner + data owner</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1397,10 +1680,26 @@
           <t>31–60 ngày</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Chứng minh chất lượng: bật trích nguồn, QA mẫu hàng tuần, thêm chuyển coach, hỗ trợ learner tại workflow</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Bật trích nguồn trong câu trả lời; QA mẫu hàng tuần; dựng đường chuyển coach; hỗ trợ learner ngay trong luồng</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>QA owner + lab coach</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ câu trả lời có nguồn và tỷ lệ hoàn thành không phải làm lại đạt mục tiêu nhóm; nếu xấu thì tăng QA và thu hẹp phạm vi</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1408,10 +1707,26 @@
           <t>61–90 ngày</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Quyết định mở rộng: so với baseline, chốt owner vận hành, kiểm tra quyền truy cập và consent, review chi phí</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>So kết quả với baseline; chốt owner vận hành; kiểm tra quyền truy cập/consent; review chi phí</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Product owner + governance owner</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ mở rộng khi chất lượng, hành vi và giá trị cùng đạt ngưỡng; nếu không thì sửa hoặc dừng pilot</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1522,12 +1837,12 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>&lt;đo hiện trạng&gt;</t>
+          <t>Đo mẫu QA tuần 1</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>&lt;mục tiêu nhóm&gt;</t>
+          <t>Đạt ngưỡng do QA owner xác nhận trước pilot</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -1537,7 +1852,7 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>&lt;tên&gt;</t>
+          <t>QA owner</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -1552,47 +1867,187 @@
           <t>Workflow</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Thời gian từ lúc mở trợ giúp đến lúc đi tiếp hoặc chuyển coach</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Đo hiện trạng</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Giảm so với baseline (không tính thời gian chờ coach là tiết kiệm)</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Log tác vụ</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Chủ quy trình</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Xem lại cách bàn giao và độ dài câu trả lời</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr"/>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Hành vi làm lại (quay lại bước cũ / hỏi lại cùng điểm)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Đo hiện trạng</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Giảm so với baseline</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Log phiên học</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Product owner</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra câu trả lời và hướng dẫn kiểm chứng</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Kết quả nghiệp vụ: tỷ lệ hoàn thành bước lab</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Baseline tuần 1</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Tăng mà không làm tăng lỗi bài tập</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Hệ thống lab / bài nộp</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Chủ nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>So sánh nhóm, điều chỉnh hoặc dừng</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr"/>
-      <c r="B10" s="7" t="inlineStr"/>
-      <c r="C10" s="7" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Rủi ro / bàn giao: tỷ lệ câu hỏi không neo được nguồn, tỷ lệ chuyển coach thành công</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Ghi hiện trạng</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Có ngưỡng cảnh báo được nhóm xác nhận</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Log lỗi và support queue</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>AI owner + coach</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung fallback, không để learner bị kẹt im lặng</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr"/>
@@ -1658,7 +2113,11 @@
           <t>Quyết định: TIẾP TỤC / SỬA / DỪNG</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>TIẾP TỤC</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1666,7 +2125,11 @@
           <t>Lý do (dựa trên bằng chứng nào)</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ câu trả lời có nguồn kiểm chứng và tỷ lệ hoàn thành không làm lại đều là chỉ số quyết định (tầng 3-4), không chỉ dựa vào lượt dùng</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1674,7 +2137,11 @@
           <t>Điều kiện / cổng kế tiếp</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ mở rộng khi chất lượng, hành vi và giá trị cùng đạt ngưỡng nhóm xác nhận ở cổng 61–90 ngày</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1682,7 +2149,11 @@
           <t>Bước tiếp theo (ai, khi nào)</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Pilot trong 1 nhóm, 1 bài lab; bổ sung fallback chuyển coach cho câu trả lời không có căn cứ; chưa rollout rộng</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1740,32 +2211,104 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr"/>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
+      <c r="A4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ số (activity vs decision)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard v1 chỉ đo lượt mở trợ giúp và thời gian tiết kiệm tự khai — không dẫn tới quyết định gì</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm phản biện A</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung chỉ số hành vi, chất lượng/tin cậy và rủi ro/bàn giao; bỏ chỉ số thời gian tiết kiệm tự khai</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Giải pháp / chia việc</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>TO-BE ở v1 chỉ thêm bước "hỏi AI" mà chưa nói rõ ai chịu trách nhiệm kết quả cuối khi AI không chắc</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm phản biện A</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Thêm cột "người chịu trách nhiệm" và "xử lý khi AI không chắc chắn" vào workflow TO-BE, gắn với Mollick</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr"/>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
+      <c r="A6" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Nguyên nhân gốc</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Nguyên nhân gốc ở v1 còn gần triệu chứng ("learner chưa quen dùng tutor"), chưa chỉ rõ vì sao</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm phản biện B</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Đào sâu bằng 5 câu hỏi chẩn đoán + ADKAR: chốt lại nguyên nhân là thiếu trích nguồn và thiếu đường chuyển coach</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
+      <c r="A7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Lộ trình</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Giai đoạn 31–60 và 61–90 ở v1 chưa có owner và dấu hiệu hoàn thành, dễ thành lịch cứng</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm phản biện B</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Gắn owner cho từng giai đoạn và định nghĩa cổng bằng ngưỡng chỉ số, không phải mốc thời gian</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>